<commit_message>
change ampli, and redac for elbow
</commit_message>
<xml_diff>
--- a/data/final/comparison_qom_long.xlsx
+++ b/data/final/comparison_qom_long.xlsx
@@ -3949,7 +3949,7 @@
         <v>0.09874276561509227</v>
       </c>
       <c r="F85">
-        <v>42030.15652531252</v>
+        <v>82796.19420993727</v>
       </c>
       <c r="G85">
         <v>10940.22335434749</v>
@@ -3961,7 +3961,7 @@
         <v>2.951758535676491</v>
       </c>
       <c r="J85">
-        <v>136.9590241187025</v>
+        <v>269.798803935129</v>
       </c>
       <c r="K85">
         <v>269.0563841784278</v>
@@ -4034,7 +4034,7 @@
         <v>31312.7936542629</v>
       </c>
       <c r="G87">
-        <v>0</v>
+        <v>11070.9608995176</v>
       </c>
       <c r="H87">
         <v>12.74505498207485</v>
@@ -4049,7 +4049,7 @@
         <v>170.2808058997619</v>
       </c>
       <c r="L87">
-        <v>0</v>
+        <v>42.37536768668815</v>
       </c>
       <c r="M87">
         <v>38.43735060712103</v>

</xml_diff>